<commit_message>
[NCBI Daily] 2026-07-15 pipeline results
</commit_message>
<xml_diff>
--- a/results/2026-07-15/NCBI_Eukaryota_Taxonomy_Summary.xlsx
+++ b/results/2026-07-15/NCBI_Eukaryota_Taxonomy_Summary.xlsx
@@ -466,10 +466,10 @@
         <v>1190</v>
       </c>
       <c r="E2" t="n">
-        <v>41926</v>
+        <v>41927</v>
       </c>
       <c r="F2" t="n">
-        <v>765268</v>
+        <v>765382</v>
       </c>
     </row>
     <row r="3">
@@ -490,10 +490,10 @@
         <v>482</v>
       </c>
       <c r="E3" t="n">
-        <v>14606</v>
+        <v>14604</v>
       </c>
       <c r="F3" t="n">
-        <v>215346</v>
+        <v>216785</v>
       </c>
     </row>
     <row r="4">
@@ -514,10 +514,10 @@
         <v>642</v>
       </c>
       <c r="E4" t="n">
-        <v>5306</v>
+        <v>5307</v>
       </c>
       <c r="F4" t="n">
-        <v>77180</v>
+        <v>77202</v>
       </c>
     </row>
     <row r="5">
@@ -541,7 +541,7 @@
         <v>1632</v>
       </c>
       <c r="F5" t="n">
-        <v>56159</v>
+        <v>56172</v>
       </c>
     </row>
     <row r="6">
@@ -565,7 +565,7 @@
         <v>4791</v>
       </c>
       <c r="F6" t="n">
-        <v>52690</v>
+        <v>52696</v>
       </c>
     </row>
     <row r="7">
@@ -589,7 +589,7 @@
         <v>1744</v>
       </c>
       <c r="F7" t="n">
-        <v>41563</v>
+        <v>41573</v>
       </c>
     </row>
     <row r="8">
@@ -637,7 +637,7 @@
         <v>4080</v>
       </c>
       <c r="F9" t="n">
-        <v>32028</v>
+        <v>32033</v>
       </c>
     </row>
     <row r="10">
@@ -661,7 +661,7 @@
         <v>1643</v>
       </c>
       <c r="F10" t="n">
-        <v>25015</v>
+        <v>25016</v>
       </c>
     </row>
     <row r="11">
@@ -733,7 +733,7 @@
         <v>1217</v>
       </c>
       <c r="F13" t="n">
-        <v>14587</v>
+        <v>14589</v>
       </c>
     </row>
     <row r="14">
@@ -757,7 +757,7 @@
         <v>308</v>
       </c>
       <c r="F14" t="n">
-        <v>12603</v>
+        <v>12605</v>
       </c>
     </row>
     <row r="15">
@@ -829,7 +829,7 @@
         <v>1167</v>
       </c>
       <c r="F17" t="n">
-        <v>11711</v>
+        <v>11712</v>
       </c>
     </row>
     <row r="18">
@@ -901,7 +901,7 @@
         <v>1428</v>
       </c>
       <c r="F20" t="n">
-        <v>10167</v>
+        <v>10168</v>
       </c>
     </row>
     <row r="21">
@@ -994,7 +994,7 @@
         <v>68</v>
       </c>
       <c r="E24" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="F24" t="n">
         <v>8346</v>
@@ -1045,7 +1045,7 @@
         <v>979</v>
       </c>
       <c r="F26" t="n">
-        <v>6994</v>
+        <v>6995</v>
       </c>
     </row>
     <row r="27">
@@ -1405,7 +1405,7 @@
         <v>524</v>
       </c>
       <c r="F41" t="n">
-        <v>2844</v>
+        <v>2845</v>
       </c>
     </row>
     <row r="42">
@@ -1429,7 +1429,7 @@
         <v>500</v>
       </c>
       <c r="F42" t="n">
-        <v>2809</v>
+        <v>2810</v>
       </c>
     </row>
     <row r="43">
@@ -1891,46 +1891,46 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mollusca</t>
+          <t>Euglenozoa</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Cephalopoda</t>
+          <t>Kinetoplastea</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D62" t="n">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="E62" t="n">
-        <v>191</v>
+        <v>57</v>
       </c>
       <c r="F62" t="n">
-        <v>1512</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Euglenozoa</t>
+          <t>Mollusca</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Kinetoplastea</t>
+          <t>Cephalopoda</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D63" t="n">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="E63" t="n">
-        <v>57</v>
+        <v>191</v>
       </c>
       <c r="F63" t="n">
         <v>1512</v>
@@ -2365,7 +2365,7 @@
         <v>53</v>
       </c>
       <c r="F81" t="n">
-        <v>952</v>
+        <v>954</v>
       </c>
     </row>
     <row r="82">
@@ -2743,7 +2743,7 @@
         <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E97" t="n">
         <v>92</v>

</xml_diff>